<commit_message>
Add ChatOps dashboard, widget session APIs, and AWS deploy prep.
Includes admin chat/leads inbox, embeddable widget updates, FastAPI dashboard routes, Redis session manager, and docker-compose for deployment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/HR-Reachout-Agent-main/WhatsApp_Leads.xlsx
+++ b/HR-Reachout-Agent-main/WhatsApp_Leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,38 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>['User is interested in learning about the services offered by the app.', 'User wants to know how to use the app effectively.', 'User has tested the app and found it awesome.', 'User is interested in a personalized demo from the team.']</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-20T03:39:56.898302</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>whatsapp_3913947408901407_1054801481058488_916206535856</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>916206535856</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ashutosh Pandey</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>aspandey1904@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>['User wants to book an appointment.', 'User has selected Monday, 25 May 2026.', 'User provided their name and email for the appointment.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: S Square WhatsApp agent, broadcast, and chattiq-wp-credits-new integration
Replace chattiq-wp-credits with chattiq-wp-credits-new and wire token tracking
into credits_store, FastAPI /credits/tokens, Express proxy, and credits UI.
Add WhatsApp flow (greeting, menu, booking, broadcast), channel admin UI,
security hardening, and remove committed deployment PEM from the repo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/HR-Reachout-Agent-main/WhatsApp_Leads.xlsx
+++ b/HR-Reachout-Agent-main/WhatsApp_Leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,38 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>['User wants to book an appointment.', 'User has selected Monday, 25 May 2026.', 'User provided their name and email for the appointment.']</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-02T18:30:21.797711</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>whatsapp_981276181065714_1072900375915131_916206535856</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>916206535856</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ashutosh Pandey</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ssquarefitnessclubpune@gmail.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>['User is interested in membership plans offered by S Square Fitness.', 'User wants to know the location of the gym.', 'User inquired about booking a visit to the gym.']</t>
         </is>
       </c>
     </row>

</xml_diff>